<commit_message>
refactor: restructure Benivo automation for deployment
</commit_message>
<xml_diff>
--- a/benivo_insert_report.xlsx
+++ b/benivo_insert_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -613,9 +613,94 @@
           <t>1008457</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
+        <is>
+          <t>{"data": {"user": {"phoneNumber": null, "gender": "", "benivoId": 603084, "firstName": "Esteban", "lastName": "test", "email": "esteban.alvarez@arrise.com"}, "assignments": [{"officeId": "d715fdb6-c93c-4940-a076-918214ca152d", "officeIdGuid": "d715fdb6-c93c-4940-a076-918214ca152d", "externalOfficeId": null, "homeCountry": null, "homeState": null, "homeCity": null, "familySize": null, "numberOfChildren": null, "includeRelocationAllowance": null, "includeMultipleAssignments": false, "policy": "Tier 1", "includeExpenseManagement": null, "assignmentJourney": "", "startDateOfAssignment": "2026-06-12T18:14:05+00:00", "endDateOfAssignment": null, "services": [], "dateOfBirth": "0001-01-01T00:00:00+00:00", "countryOfBirth": null, "departureCity": "", "departureCountry": "", "hostCountry": null, "mobilitySpecialistEmail": null, "hiringManagerName": null, "hiringManagerEmail": null, "repatriationStatus": "None", "dependents": [], "passports": [], "homeResidentialAddresses": [], "hostResidentialAddresses": [], "assignmentExtensions": [], "hostBusinessUnit": null, "hostJobRole": null, "employeeID": null, "assignmentNotes": null, "hostCostCentre": null, "billingEntity": null, "policyType": null, "externalAssignmentID": null, "assignmentType": null, "hostLegalEntity": null, "generalLedgerCode": null, "relocatingWith": null, "status": "Created", "talentProfile": false, "confidentialMove": false, "maritalStatus": null, "hostAnnualNetSalary": null, "hostAnnualNetSalaryCurrency": null, "homeAnnualNetSalary": null, "homeAnnualNetSalaryCurrency": null, "hostAnnualTotalCompensation": null, "hostAnnualTotalCompensationCurrency": null, "homeJobRole": null, "homeCostCentre": null, "hostJobRoleType": null, "hostJobRoleSchedule": null, "homeBusinessUnit": null, "numberOfDependentsNotTravelling": null, "mobilityReason": null, "hostJobDescription": null, "hostJobRoleCertificationType": null, "hostJobRoleRegulated": null, "hostJobRoleStatus": null, "relocatingWithDirectReports": null, "isHostCostCentreNew": null, "hostJobLevel": null, "homeJobLevel": null, "homeWorkAddress": null, "hostBusinessUnit2": null, "hostBusinessUnit3": null, "hostBusinessUnit4": null, "hostBusinessUnit5": null, "hostBusinessUnit6": null, "hostBusinessUnit7": null, "hrContactName": null, "hrContactEmail": null, "hostAnnualBaseSalaryCurrency": null, "hostAnnualBaseSalary": null, "immigrationApproved": null, "hrContactName2": null, "hrContactEmail2": null, "hrRecruiterName": null, "hrRecruiterEmail": null, "candidateId": null, "secondaryEmployeeType": null, "hrContactName3": null, "hrContactEmail3": null, "employeeRoleType": null, "secondaryEmployeeRoleType": null, "companySystemId": null, "immigrationRequired": null, "secondaryPolicyType": null, "employeeAlias": null, "hostPositionId": null, "homeLegalEntity": null, "hostSecondaryJobLevel": null, "payGroup": null, "payrollType": null, "homeCountryHousingStatus": null, "hostCompanyCode": null, "hireType": null, "hostStrategicBusinessUnit": null, "fixedTermContractEndDate": null, "homeOrgLevel2": null, "homeOrgLevel3": null, "homeOrgLevel4": null, "hostOrgLevel2": null, "hostManagerEmployeeID": null, "mobilityType": null, "hostCostCentreDropdown": null, "homeBusinessUnitDropdown": null, "hostBusinessUnitDropdown": null, "hostLegalEntityDropdown": null, "homeLegalEntityDropdown": null, "chargeableCostCentre": null, "proposedStartDate": null, "budgetApproverName": null, "budgetApproverEmail": null, "chargeableCostCentre2": null, "terminationDate": null, "businessCase": null, "homeLegalEntityCode": null, "hostDepartment": null, "hostDepartmentDropdown": null, "homeDepartment": null, "lumpSumAmount": null, "hostPositionId2": null, "socialSecurityCertificateType": null, "lastSalaryReviewDate": null, "assessmentOutcomePwd": null, "assessmentOutcomeTax": null, "assessmentOutcomeSocialSecurity": null, "assessmentOutcomeImmigration": null, "pensionFundType": null, "customDropdown1": null, "internshipType": null, "fileNumber": null, "educationLevel": null, "visaStartDate": null, "visaEndDate": null, "certificateOfCoverageStartDate": null, "certificateOfCoverageEndDate": null, "endOfAssignmentCity": null, "relocationPhase": null, "homeAnnualBaseSalaryCurrency": null, "homeAnnualBaseSalary": null, "homeAnnualTotalCompensationCurrency": null, "homeAnnualTotalCompensation": null, "homeBonusCurrency": null, "homeBonus": null, "hostBonusCurrency": null, "hostBonus": null, "homeSecondaryJobLevel": null, "customCostCenter1": null, "customCostCenter2": null, "customCostCenterName1": null, "customCostCenterName2": null, "employmentStatusAtRelocationStart": null, "jobLocationType": null, "jobOpeningType": null, "mobilityDrivenBy": null, "primaryMobilityType": null, "projectAssigned": null, "variationReferenceId": null, "activities": null, "employeeContractStatus": null, "contractType": null, "contractStartDate": null, "seniorityDate": null, "homePositionId": null, "homeJobCode": null, "postedWorkerNotificationStartDate": null, "posted</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-12T19:04:04Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ALREADY_EXISTS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NO_APPLIES</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>esteban.alvarez@arrise.com</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Esteban</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Colombia (Live Casino)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>d715fdb6-c93c-4940-a076-918214ca152d</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-06-12T19:04:12Z</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>603084</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1008457</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
         <is>
           <t>{"data": {"user": {"phoneNumber": null, "gender": "", "benivoId": 603084, "firstName": "Esteban", "lastName": "test", "email": "esteban.alvarez@arrise.com"}, "assignments": [{"officeId": "d715fdb6-c93c-4940-a076-918214ca152d", "officeIdGuid": "d715fdb6-c93c-4940-a076-918214ca152d", "externalOfficeId": null, "homeCountry": null, "homeState": null, "homeCity": null, "familySize": null, "numberOfChildren": null, "includeRelocationAllowance": null, "includeMultipleAssignments": false, "policy": "Tier 1", "includeExpenseManagement": null, "assignmentJourney": "", "startDateOfAssignment": "2026-06-12T18:14:05+00:00", "endDateOfAssignment": null, "services": [], "dateOfBirth": "0001-01-01T00:00:00+00:00", "countryOfBirth": null, "departureCity": "", "departureCountry": "", "hostCountry": null, "mobilitySpecialistEmail": null, "hiringManagerName": null, "hiringManagerEmail": null, "repatriationStatus": "None", "dependents": [], "passports": [], "homeResidentialAddresses": [], "hostResidentialAddresses": [], "assignmentExtensions": [], "hostBusinessUnit": null, "hostJobRole": null, "employeeID": null, "assignmentNotes": null, "hostCostCentre": null, "billingEntity": null, "policyType": null, "externalAssignmentID": null, "assignmentType": null, "hostLegalEntity": null, "generalLedgerCode": null, "relocatingWith": null, "status": "Created", "talentProfile": false, "confidentialMove": false, "maritalStatus": null, "hostAnnualNetSalary": null, "hostAnnualNetSalaryCurrency": null, "homeAnnualNetSalary": null, "homeAnnualNetSalaryCurrency": null, "hostAnnualTotalCompensation": null, "hostAnnualTotalCompensationCurrency": null, "homeJobRole": null, "homeCostCentre": null, "hostJobRoleType": null, "hostJobRoleSchedule": null, "homeBusinessUnit": null, "numberOfDependentsNotTravelling": null, "mobilityReason": null, "hostJobDescription": null, "hostJobRoleCertificationType": null, "hostJobRoleRegulated": null, "hostJobRoleStatus": null, "relocatingWithDirectReports": null, "isHostCostCentreNew": null, "hostJobLevel": null, "homeJobLevel": null, "homeWorkAddress": null, "hostBusinessUnit2": null, "hostBusinessUnit3": null, "hostBusinessUnit4": null, "hostBusinessUnit5": null, "hostBusinessUnit6": null, "hostBusinessUnit7": null, "hrContactName": null, "hrContactEmail": null, "hostAnnualBaseSalaryCurrency": null, "hostAnnualBaseSalary": null, "immigrationApproved": null, "hrContactName2": null, "hrContactEmail2": null, "hrRecruiterName": null, "hrRecruiterEmail": null, "candidateId": null, "secondaryEmployeeType": null, "hrContactName3": null, "hrContactEmail3": null, "employeeRoleType": null, "secondaryEmployeeRoleType": null, "companySystemId": null, "immigrationRequired": null, "secondaryPolicyType": null, "employeeAlias": null, "hostPositionId": null, "homeLegalEntity": null, "hostSecondaryJobLevel": null, "payGroup": null, "payrollType": null, "homeCountryHousingStatus": null, "hostCompanyCode": null, "hireType": null, "hostStrategicBusinessUnit": null, "fixedTermContractEndDate": null, "homeOrgLevel2": null, "homeOrgLevel3": null, "homeOrgLevel4": null, "hostOrgLevel2": null, "hostManagerEmployeeID": null, "mobilityType": null, "hostCostCentreDropdown": null, "homeBusinessUnitDropdown": null, "hostBusinessUnitDropdown": null, "hostLegalEntityDropdown": null, "homeLegalEntityDropdown": null, "chargeableCostCentre": null, "proposedStartDate": null, "budgetApproverName": null, "budgetApproverEmail": null, "chargeableCostCentre2": null, "terminationDate": null, "businessCase": null, "homeLegalEntityCode": null, "hostDepartment": null, "hostDepartmentDropdown": null, "homeDepartment": null, "lumpSumAmount": null, "hostPositionId2": null, "socialSecurityCertificateType": null, "lastSalaryReviewDate": null, "assessmentOutcomePwd": null, "assessmentOutcomeTax": null, "assessmentOutcomeSocialSecurity": null, "assessmentOutcomeImmigration": null, "pensionFundType": null, "customDropdown1": null, "internshipType": null, "fileNumber": null, "educationLevel": null, "visaStartDate": null, "visaEndDate": null, "certificateOfCoverageStartDate": null, "certificateOfCoverageEndDate": null, "endOfAssignmentCity": null, "relocationPhase": null, "homeAnnualBaseSalaryCurrency": null, "homeAnnualBaseSalary": null, "homeAnnualTotalCompensationCurrency": null, "homeAnnualTotalCompensation": null, "homeBonusCurrency": null, "homeBonus": null, "hostBonusCurrency": null, "hostBonus": null, "homeSecondaryJobLevel": null, "customCostCenter1": null, "customCostCenter2": null, "customCostCenterName1": null, "customCostCenterName2": null, "employmentStatusAtRelocationStart": null, "jobLocationType": null, "jobOpeningType": null, "mobilityDrivenBy": null, "primaryMobilityType": null, "projectAssigned": null, "variationReferenceId": null, "activities": null, "employeeContractStatus": null, "contractType": null, "contractStartDate": null, "seniorityDate": null, "homePositionId": null, "homeJobCode": null, "postedWorkerNotificationStartDate": null, "posted</t>
         </is>

</xml_diff>